<commit_message>
Expand GateSignal evidence and unify the suite
</commit_message>
<xml_diff>
--- a/examples/gatesignal-blank-template.xlsx
+++ b/examples/gatesignal-blank-template.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Cash flows" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Volume bridge" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Risks" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Challenge" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Brand evidence" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Challenge" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Metadata'!$A$1:$B$7</definedName>
@@ -20,7 +21,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cash flows'!$A$1:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volume bridge'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Risks'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Challenge'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Brand evidence'!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Challenge'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -958,6 +960,311 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>claim_or_risk</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>evidence_direction</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>evidence_strength</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>materiality</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>must_resolve</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>evidence_note</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>next_test</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Category fit</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>The proposed category use is credible for the focal brand</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Image and value fit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Brand meanings and customer expectations fit the offer or partner</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Transfer asymmetry</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Positive associations transfer in both directions without one party carrying most downside</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dilution and confusion</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>The extension or alliance will not blur, weaken, or contradict core brand meaning</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Control and governance</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Rights, quality control, exit, data use, and incident authority are explicit</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Disclosure</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Customers can recognize the commercial relationship and material claims</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Activism</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Public positions are congruent with behavior, stakeholder expectations, and partner conduct</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Reputation spillover</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Partner, category, and controversy spillovers have an owned response and exit path</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Not assessed</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>